<commit_message>
fix(content): align policy copy and source materials
</commit_message>
<xml_diff>
--- a/curriculum/unit_8_grants/phoenix_ai_grants_handbook.xlsx
+++ b/curriculum/unit_8_grants/phoenix_ai_grants_handbook.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="👑 補助素材盤點與套利規畫" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="📊 補助匹配與風險矩陣" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="✍️ 計畫書 7 大核心骨架" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="📅 月度執行與風險追蹤" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="📋 結案核銷 20 點自評檢核" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="👑 補助素材盤點與資源匹配規劃" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 補助匹配與風險矩陣" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="✍️ 計畫書 7 大核心骨架" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 月度執行與風險追蹤" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📋 結案核銷 20 點自評檢核" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -140,7 +140,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -162,11 +162,104 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -258,6 +351,15 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -635,7 +737,7 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>鳳凰 AI 補助潛在素材盤點與多層次套利規劃表</t>
+          <t>鳳凰 AI 補助潛在素材盤點與多層次政策工具組合規劃表</t>
         </is>
       </c>
     </row>
@@ -758,11 +860,10 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>【Part B：多層次政策工具組合套利（以 NT$ 800 萬智慧檢測研發專案為例）】</t>
+          <t>【Part B：多層次政策工具組合（以 NT$ 800 萬智慧檢測研發專案為例）】</t>
         </is>
       </c>
     </row>
@@ -774,9 +875,11 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>套利說明 / 效益金額</t>
-        </is>
-      </c>
+          <t>效益說明 / 效益金額</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="36" t="n"/>
     </row>
     <row r="12" ht="35" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -789,8 +892,8 @@
           <t>獲得 50% 資金補貼 (NT$ 4,000,000)</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
+      <c r="C12" s="35" t="n"/>
+      <c r="D12" s="36" t="n"/>
     </row>
     <row r="13" ht="35" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -803,8 +906,8 @@
           <t>智慧機械與 AI 系統購置支出之 5% 抵減營所稅 (以軟硬體購置費 NT$ 2,000,000 計算，可直接抵減 NT$ 100,000 稅額)</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="36" t="n"/>
     </row>
     <row r="14" ht="35" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -817,8 +920,8 @@
           <t>員工內訓講師與場地費 100% 全額補助 (NT$ 150,000)</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="36" t="n"/>
     </row>
     <row r="15" ht="35" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -831,14 +934,13 @@
           <t>免除內部找尋教授的行政摩擦，取得審查額外加分 5-10%</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-    </row>
-    <row r="16"/>
+      <c r="C15" s="35" t="n"/>
+      <c r="D15" s="36" t="n"/>
+    </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>📊 套利後實質成效精算（NT$ 800 萬專案）</t>
+          <t>📊 組合後實質成效精算（NT$ 800 萬專案）</t>
         </is>
       </c>
     </row>
@@ -853,6 +955,8 @@
           <t>金額 (NT$)</t>
         </is>
       </c>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="36" t="n"/>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -865,8 +969,8 @@
           <t>8,000,000</t>
         </is>
       </c>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
+      <c r="C19" s="35" t="n"/>
+      <c r="D19" s="36" t="n"/>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -879,8 +983,8 @@
           <t>4,000,000</t>
         </is>
       </c>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
+      <c r="C20" s="35" t="n"/>
+      <c r="D20" s="36" t="n"/>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -893,8 +997,8 @@
           <t>100,000</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
+      <c r="C21" s="35" t="n"/>
+      <c r="D21" s="36" t="n"/>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -907,8 +1011,8 @@
           <t>150,000</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="11" t="n"/>
+      <c r="C22" s="35" t="n"/>
+      <c r="D22" s="36" t="n"/>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
@@ -921,10 +1025,9 @@
           <t>3,750,000 (自籌比例自 100% 降至 46.8%！)</t>
         </is>
       </c>
-      <c r="C23" s="15" t="n"/>
-      <c r="D23" s="15" t="n"/>
-    </row>
-    <row r="24"/>
+      <c r="C23" s="35" t="n"/>
+      <c r="D23" s="36" t="n"/>
+    </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
@@ -943,6 +1046,8 @@
           <t>對接狀態 / 說明</t>
         </is>
       </c>
+      <c r="C26" s="35" t="n"/>
+      <c r="D26" s="36" t="n"/>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
@@ -955,8 +1060,8 @@
           <t>[ ] 預定合作學術機構（提供學術正統性加分）</t>
         </is>
       </c>
-      <c r="C27" s="16" t="n"/>
-      <c r="D27" s="16" t="n"/>
+      <c r="C27" s="35" t="n"/>
+      <c r="D27" s="36" t="n"/>
     </row>
     <row r="28" ht="25" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
@@ -969,8 +1074,8 @@
           <t>[ ] 預定合作學術機構</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="11" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="36" t="n"/>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
@@ -983,8 +1088,8 @@
           <t>[ ] 預定法人聯合輔導窗口（中南部傳產製造業主要對接窗口）</t>
         </is>
       </c>
-      <c r="C29" s="16" t="n"/>
-      <c r="D29" s="16" t="n"/>
+      <c r="C29" s="35" t="n"/>
+      <c r="D29" s="36" t="n"/>
     </row>
     <row r="30" ht="25" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
@@ -997,8 +1102,8 @@
           <t>[ ] 預定法人聯合輔導窗口</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
+      <c r="C30" s="35" t="n"/>
+      <c r="D30" s="36" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -1190,7 +1295,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="25" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -1209,8 +1313,8 @@
           <t>【極佳匹配】項目可行性極高，專案團隊可即刻著手撰寫計畫書並進行申報！</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
+      <c r="C12" s="35" t="n"/>
+      <c r="D12" s="36" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
@@ -1223,8 +1327,8 @@
           <t>【黃色預警】部分指標存在潛在風險（如現金流或工時）。建議修正 KPI 指標、調整預算編列或縮短執行期，再送件。</t>
         </is>
       </c>
-      <c r="C13" s="27" t="n"/>
-      <c r="D13" s="27" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="36" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="28" t="inlineStr">
@@ -1237,8 +1341,8 @@
           <t>【紅色否決】風險過高（如團隊不穩或自籌款嚴重不足）。極易結案失敗或被追回補助款，不建議在現有架構下申請。</t>
         </is>
       </c>
-      <c r="C14" s="29" t="n"/>
-      <c r="D14" s="29" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="36" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1283,21 +1387,19 @@
 3. 潛規則 3 (KPI 80% 安全防護)：效益指標（如良率提升）承諾實際預估值的 80% 即可，確保結案順利甚至超標，防範被追回款項。</t>
         </is>
       </c>
-      <c r="B2" s="31" t="n"/>
-      <c r="C2" s="31" t="n"/>
-      <c r="D2" s="31" t="n"/>
+      <c r="B2" s="37" t="n"/>
+      <c r="C2" s="37" t="n"/>
+      <c r="D2" s="38" t="n"/>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="31" t="n"/>
-      <c r="B3" s="31" t="n"/>
-      <c r="C3" s="31" t="n"/>
-      <c r="D3" s="31" t="n"/>
+      <c r="A3" s="39" t="n"/>
+      <c r="D3" s="40" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="31" t="n"/>
-      <c r="B4" s="31" t="n"/>
-      <c r="C4" s="31" t="n"/>
-      <c r="D4" s="31" t="n"/>
+      <c r="A4" s="41" t="n"/>
+      <c r="B4" s="42" t="n"/>
+      <c r="C4" s="42" t="n"/>
+      <c r="D4" s="43" t="n"/>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1458,7 +1560,7 @@
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>專案總預算編列新台幣 800 萬元。其中：(1) 研發人事費：編列 NT$ 440 萬（55%，符合人事費不超 60% 限制）；(2) 消耗性器材與材料費：編列 NT$ 80 萬（10%，用於雲端 GPU 訓練 Token 費與測試模具耗損）；(3) 學研與委外開發費：委託高科大產學合作編列 NT$ 160 萬（20%）；(4) 研發設備使用折舊費：購置地端伺服器與 Edge AI 卡編列 NT$ 120 萬（15%）。此購置設備同時向財政部申請「產業創新條例第 10 條之 1」智慧機械與 AI 系統抵減，預計可享 5% 營所稅抵減（NT$ 6 萬元），實現多重政策套利。</t>
+          <t>專案總預算編列新台幣 800 萬元。其中：(1) 研發人事費：編列 NT$ 440 萬（55%，符合人事費不超 60% 限制）；(2) 消耗性器材與材料費：編列 NT$ 80 萬（10%，用於雲端 GPU 訓練 Token 費與測試模具耗損）；(3) 學研與委外開發費：委託高科大產學合作編列 NT$ 160 萬（20%）；(4) 研發設備使用折舊費：購置地端伺服器與 Edge AI 卡編列 NT$ 120 萬（15%）。此購置設備同時向財政部申請「產業創新條例第 10 條之 1」智慧機械與 AI 系統抵減，預計可享 5% 營所稅抵減（NT$ 6 萬元），實現多重政策資源規劃。</t>
         </is>
       </c>
     </row>
@@ -1543,8 +1645,8 @@
           <t>【模組 1：技術里程碑與 Gantt Chart 進度查核】</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n"/>
-      <c r="C3" s="11" t="n"/>
+      <c r="B3" s="35" t="n"/>
+      <c r="C3" s="36" t="n"/>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="33" t="inlineStr">
@@ -1593,8 +1695,8 @@
           <t>【模組 2：台灣勞基法與研發工時防護欄 (🚨 審計稽核最大紅線)】</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
+      <c r="B7" s="35" t="n"/>
+      <c r="C7" s="36" t="n"/>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="33" t="inlineStr">
@@ -1654,8 +1756,8 @@
           <t>【模組 3：AI/MLOps 模型健康與資料合規追蹤】</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
+      <c r="B12" s="35" t="n"/>
+      <c r="C12" s="36" t="n"/>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="34" t="inlineStr">
@@ -1759,9 +1861,9 @@
           <t>一、財務、發票與會計科目合規 (Financial &amp; Invoices)</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n"/>
-      <c r="C3" s="11" t="n"/>
-      <c r="D3" s="11" t="n"/>
+      <c r="B3" s="35" t="n"/>
+      <c r="C3" s="35" t="n"/>
+      <c r="D3" s="36" t="n"/>
     </row>
     <row r="4" ht="35" customHeight="1">
       <c r="A4" s="33" t="inlineStr">
@@ -1879,9 +1981,9 @@
           <t>二、人力資源、薪資與工時憑證 (HR &amp; Attendance)</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
+      <c r="B9" s="35" t="n"/>
+      <c r="C9" s="35" t="n"/>
+      <c r="D9" s="36" t="n"/>
     </row>
     <row r="10" ht="35" customHeight="1">
       <c r="A10" s="33" t="inlineStr">
@@ -1999,9 +2101,9 @@
           <t>三、設備、財產登記與資安防護 (Equipment &amp; Security)</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
+      <c r="B15" s="35" t="n"/>
+      <c r="C15" s="35" t="n"/>
+      <c r="D15" s="36" t="n"/>
     </row>
     <row r="16" ht="35" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
@@ -2119,9 +2221,9 @@
           <t>四、技術 KPI 指標、成果展示與佐證 (Technical KPIs &amp; Demo)</t>
         </is>
       </c>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
+      <c r="B21" s="35" t="n"/>
+      <c r="C21" s="35" t="n"/>
+      <c r="D21" s="36" t="n"/>
     </row>
     <row r="22" ht="35" customHeight="1">
       <c r="A22" s="33" t="inlineStr">

</xml_diff>